<commit_message>
Refocus product backlog on editing receipt entries
Reprioritize user stories based on the Lab 2 proposal feedback to focus
on categorizing, editing details, and generating summary views. Photo
capture and account features move to lower priorities. Document the MVP
scope as all priority 1 and 2 user stories across three windows.
</commit_message>
<xml_diff>
--- a/documentation/Product_Backlog.xlsx
+++ b/documentation/Product_Backlog.xlsx
@@ -43,12 +43,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>take a picture of a receipt</t>
+          <t>add a receipt entry with a vendor, date, and amount</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>I can capture proof of a purchase quickly</t>
+          <t>I can record a purchase I made</t>
         </is>
       </c>
     </row>
@@ -63,12 +63,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>save a receipt photo as an expense</t>
+          <t>view my list of receipt entries</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>I can track spending without typing everything from scratch</t>
+          <t>I can see all purchases I have recorded</t>
         </is>
       </c>
     </row>
@@ -83,12 +83,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>view my receipt photos</t>
+          <t>edit the details of a receipt entry</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>I can find a purchase I already captured</t>
+          <t>I can correct mistakes in a recorded purchase</t>
         </is>
       </c>
     </row>
@@ -103,12 +103,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>choose a category for a receipt expense</t>
+          <t>assign a category to a receipt entry</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>I can organize where money is going</t>
+          <t>I can organize where my money is going</t>
         </is>
       </c>
     </row>
@@ -123,18 +123,18 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>delete a receipt expense</t>
+          <t>mark a receipt entry as tax-related</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>I can remove a capture I do not need</t>
+          <t>I can identify business costs for tax time</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -143,12 +143,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>create an account</t>
+          <t>delete a receipt entry</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>I can keep my business receipts saved privately</t>
+          <t>I can remove a purchase I no longer need to track</t>
         </is>
       </c>
     </row>
@@ -163,12 +163,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>log in to my account</t>
+          <t>view total spending for each category</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>I can access my receipt expenses securely</t>
+          <t>I can see which areas of the business cost the most</t>
         </is>
       </c>
     </row>
@@ -183,12 +183,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>update my credentials</t>
+          <t>view total spending within a date range</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>I can keep my account secure</t>
+          <t>I can review a month or quarter of purchases</t>
         </is>
       </c>
     </row>
@@ -203,18 +203,18 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>delete my account</t>
+          <t>view the total of tax-related receipt entries</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>I can remove my information from the system</t>
+          <t>I know how much to report for tax preparation</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -223,18 +223,18 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>confirm or edit the amount on a receipt expense</t>
+          <t>filter receipt entries by category</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>I can make sure the saved total is correct</t>
+          <t>I can review purchases in one area of the business</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -243,12 +243,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>mark a receipt expense as tax-related</t>
+          <t>add a short note to a receipt entry</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>I can prepare business costs for tax time</t>
+          <t>I can remember the business purpose of a purchase</t>
         </is>
       </c>
     </row>
@@ -263,18 +263,18 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>view expenses created from receipt photos</t>
+          <t>save my receipt entries to a file</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>I can see my spending history in one place</t>
+          <t>I keep my records between uses of the application</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -283,18 +283,18 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>filter receipt expenses by category</t>
+          <t>export tax-related receipt entries to a file</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>I can see spending in one area of the business</t>
+          <t>I can share a tax-ready list with my tax preparer</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -303,18 +303,18 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>filter receipt expenses by date range</t>
+          <t>attach a photo of the receipt to a receipt entry</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>I can review a month or quarter of purchases</t>
+          <t>I keep proof of each purchase</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -323,18 +323,18 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>view total spending from receipt expenses this month</t>
+          <t>take a picture of a receipt</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>I can understand current business costs</t>
+          <t>I can capture proof of a purchase quickly</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -343,18 +343,18 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>view only tax-related receipt expenses</t>
+          <t>create an account</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>I can focus on records needed for tax preparation</t>
+          <t>I can keep my business receipts private</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -363,18 +363,18 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>add a short note to a receipt expense</t>
+          <t>log in to my account</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>I can remember the business purpose of the purchase</t>
+          <t>I can access my receipt entries securely</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -383,18 +383,18 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>retake or replace a receipt photo</t>
+          <t>update my credentials</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>I can fix a blurry or incomplete picture</t>
+          <t>I can keep my account secure</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -403,18 +403,18 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>export receipt expenses to a file</t>
+          <t>delete my account</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>I can share a clean list with a bookkeeper or tax preparer</t>
+          <t>I can remove my information from the system</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -423,12 +423,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>export tax-related receipt expenses only</t>
+          <t>have receipt details suggested from a photo</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>I can create a tax-ready expense report</t>
+          <t>I spend less time entering vendors and amounts</t>
         </is>
       </c>
     </row>
@@ -438,57 +438,24 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>have receipt details suggested from the photo</t>
+          <t>deactivate a user account</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>I can spend even less time entering amounts and vendors</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23">
-        <v>5</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>get a reminder to photograph receipts I marked incomplete</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>I can finish capturing proof before tax time</t>
+          <t>I can stop access for someone who should no longer use the system</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24">
-        <v>5</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Admin</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>deactivate a user account</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>I can stop access for someone who should no longer use the system</t>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>MVP Scope: all priority 1 and 2 user stories</t>
         </is>
       </c>
     </row>

</xml_diff>